<commit_message>
Populate Cover & Instructions tab with Sectra metadata (4 fields pending verification)
Stage 3 Phase 2A: complete Cover & Instructions tab with company identifiers (Sectra AB, SECT B, Nasdaq Stockholm Large Cap), reporting metadata (IFRS, SEK Millions, FY May-April), source documentation (investor.sectra.com primary).

Four market/analyst assumptions entered with tentative values pending verification:
- Tax Rate 20.6% (Sweden statutory; effective rate to verify from Income Statement extraction)
- Cost of Capital 8.0% (class working WACC; refine in Stage 4 if instructor provides different default)
- Share Price SEK 320 (estimated April 30, 2025 close; verify Yahoo Finance historical SECT-B.ST)
- Shares Outstanding 192.67M (per S&P Global; verify FY24/25 Annual Report share capital note)

Next: populate Income Statement (Phase 3), Balance Sheet (Phase 4), Cash Flow (Phase 5). Will refine tentative values during/after statement extraction.
</commit_message>
<xml_diff>
--- a/models/builds/2026-05-17-cam-sectra-financials.xlsx
+++ b/models/builds/2026-05-17-cam-sectra-financials.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\shidler\docs\templates\spreadsheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\0.BUS Finance\Corporate-Finance\models\builds\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_C2087B7F3B7CCEACD4328DE2D1E5418A185D2F1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D20585A8-810B-4F25-B611-C4263D13F694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1905" yWindow="480" windowWidth="13065" windowHeight="15345" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -109,7 +109,7 @@
     <definedName name="yearCurrent">Ratios!$C$6</definedName>
     <definedName name="yearStart">Ratios!$C$7</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -127,7 +127,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="324">
   <si>
     <t>Ratios &amp; Derived Inputs</t>
   </si>
@@ -993,63 +993,36 @@
     <t>Company</t>
   </si>
   <si>
-    <t>[Your Company Name]</t>
-  </si>
-  <si>
     <t>Ticker</t>
   </si>
   <si>
-    <t>[TICKER]</t>
-  </si>
-  <si>
     <t>Industry</t>
   </si>
   <si>
-    <t>[Industry]</t>
-  </si>
-  <si>
     <t>Fiscal Year (current)</t>
   </si>
   <si>
-    <t>[FYYYYY]</t>
-  </si>
-  <si>
     <t>Fiscal Year (prior)</t>
   </si>
   <si>
     <t>Data Source</t>
   </si>
   <si>
-    <t>[SEC EDGAR 10-K URL / Yahoo Finance / etc.]</t>
-  </si>
-  <si>
     <t>Units</t>
   </si>
   <si>
     <t>Tax Rate</t>
   </si>
   <si>
-    <t>[Statutory 21% / Effective rate from financials — and why]</t>
-  </si>
-  <si>
     <t>Cost of Capital</t>
   </si>
   <si>
-    <t>[X.X% — source/method, e.g., CAPM, class working WACC]</t>
-  </si>
-  <si>
     <t>Share Price</t>
   </si>
   <si>
-    <t>[FY-end closing price]</t>
-  </si>
-  <si>
     <t>Shares Outstanding</t>
   </si>
   <si>
-    <t>[M shares — diluted weighted avg]</t>
-  </si>
-  <si>
     <t>BUS-629 Project Use</t>
   </si>
   <si>
@@ -1093,6 +1066,39 @@
   </si>
   <si>
     <t>Du Pont ROE (Ratios!C76) will not exactly equal direct ROE (Ratios!C49) in this model: the leverage component uses current-year balances while asset turnover uses prior-year assets. Explain this time-mismatch in your Stage 4 memo.</t>
+  </si>
+  <si>
+    <t>Sectra AB (publ)</t>
+  </si>
+  <si>
+    <t>SECT B</t>
+  </si>
+  <si>
+    <t>Healthcare IT — Medical Imaging &amp; Secure Communications</t>
+  </si>
+  <si>
+    <t>FY2024/2025 (ending April 30, 2025)</t>
+  </si>
+  <si>
+    <t>FY2023/2024 (ending April 30, 2024)</t>
+  </si>
+  <si>
+    <t>investor.sectra.com (Annual Reports FY24/25 and FY23/24, IFRS-audited)</t>
+  </si>
+  <si>
+    <t>All figures in SEK millions unless otherwise noted</t>
+  </si>
+  <si>
+    <t>20.6% (Sweden statutory corporate income tax rate, effective since 2021; effective rate may differ — verify from Sectra Income Statement)</t>
+  </si>
+  <si>
+    <t>8.0% — class working WACC (BUS-629 default; refine in Stage 4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> SEK 320 (estimated close April 30, 2025 — verify Yahoo Finance historical SECT-B.ST)</t>
+  </si>
+  <si>
+    <t>192.67 million (per Sectra IR / S&amp;P Global; verify FY24/25 Annual Report share note)</t>
   </si>
 </sst>
 </file>
@@ -1222,7 +1228,7 @@
       <name val="Open Sans"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1265,6 +1271,12 @@
         <bgColor rgb="FFE6F2EF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1293,7 +1305,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1373,7 +1385,7 @@
     <xf numFmtId="49" fontId="18" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1381,7 +1393,11 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1685,7 +1701,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:C41"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -1693,39 +1709,39 @@
     <col min="4" max="4" width="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="8" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:3" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B4" s="51" t="s">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="45" t="s">
         <v>157</v>
       </c>
       <c r="C4" s="46"/>
     </row>
-    <row r="5" spans="2:3" ht="26" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="5" spans="2:3" ht="26.1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="49" t="s">
         <v>158</v>
       </c>
       <c r="C5" s="46"/>
     </row>
-    <row r="6" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="6" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="47" t="s">
         <v>159</v>
       </c>
       <c r="C6" s="46"/>
     </row>
-    <row r="7" spans="2:3" ht="4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:3" ht="3.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
     </row>
-    <row r="9" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="48" t="s">
         <v>160</v>
       </c>
       <c r="C9" s="46"/>
     </row>
-    <row r="10" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>161</v>
       </c>
@@ -1733,7 +1749,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
         <v>163</v>
       </c>
@@ -1741,7 +1757,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="12" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
         <v>165</v>
       </c>
@@ -1749,7 +1765,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="13" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
         <v>167</v>
       </c>
@@ -1757,7 +1773,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="14" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
         <v>169</v>
       </c>
@@ -1765,7 +1781,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="15" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
         <v>171</v>
       </c>
@@ -1773,13 +1789,13 @@
         <v>172</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="48" t="s">
         <v>173</v>
       </c>
       <c r="C17" s="46"/>
     </row>
-    <row r="18" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="5" t="s">
         <v>174</v>
       </c>
@@ -1787,7 +1803,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="6" t="s">
         <v>176</v>
       </c>
@@ -1795,7 +1811,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="20" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="8" t="s">
         <v>178</v>
       </c>
@@ -1803,7 +1819,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="21" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="9" t="s">
         <v>180</v>
       </c>
@@ -1811,7 +1827,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="22" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="10" t="s">
         <v>182</v>
       </c>
@@ -1819,13 +1835,13 @@
         <v>183</v>
       </c>
     </row>
-    <row r="24" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="48" t="s">
         <v>184</v>
       </c>
       <c r="C24" s="46"/>
     </row>
-    <row r="25" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="5" t="s">
         <v>185</v>
       </c>
@@ -1833,7 +1849,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="26" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="11" t="s">
         <v>186</v>
       </c>
@@ -1841,7 +1857,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="27" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="11" t="s">
         <v>188</v>
       </c>
@@ -1849,7 +1865,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="28" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="11" t="s">
         <v>190</v>
       </c>
@@ -1857,7 +1873,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="29" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="11" t="s">
         <v>192</v>
       </c>
@@ -1865,7 +1881,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="30" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="11" t="s">
         <v>194</v>
       </c>
@@ -1873,7 +1889,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="31" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="11" t="s">
         <v>196</v>
       </c>
@@ -1881,7 +1897,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="32" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="11" t="s">
         <v>198</v>
       </c>
@@ -1889,7 +1905,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="33" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="11" t="s">
         <v>200</v>
       </c>
@@ -1897,13 +1913,13 @@
         <v>201</v>
       </c>
     </row>
-    <row r="36" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="48" t="s">
         <v>202</v>
       </c>
       <c r="C36" s="46"/>
     </row>
-    <row r="37" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="12" t="s">
         <v>203</v>
       </c>
@@ -1911,7 +1927,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="38" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="12" t="s">
         <v>205</v>
       </c>
@@ -1919,7 +1935,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41" s="50" t="s">
         <v>207</v>
       </c>
@@ -1943,7 +1959,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:H23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
@@ -1953,17 +1969,17 @@
     <col min="7" max="8" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" ht="23" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="2" spans="2:8" ht="23.1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="14" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="5" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="16" t="s">
         <v>210</v>
       </c>
@@ -1983,7 +1999,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="18" t="s">
         <v>214</v>
       </c>
@@ -1991,7 +2007,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="12" t="s">
         <v>216</v>
       </c>
@@ -2003,7 +2019,7 @@
       <c r="G7" s="19"/>
       <c r="H7" s="19"/>
     </row>
-    <row r="8" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12" t="s">
         <v>218</v>
       </c>
@@ -2015,7 +2031,7 @@
       <c r="G8" s="19"/>
       <c r="H8" s="19"/>
     </row>
-    <row r="9" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
         <v>220</v>
       </c>
@@ -2027,7 +2043,7 @@
       <c r="G9" s="19"/>
       <c r="H9" s="19"/>
     </row>
-    <row r="10" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="12" t="s">
         <v>222</v>
       </c>
@@ -2045,7 +2061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="20" t="s">
         <v>224</v>
       </c>
@@ -2058,14 +2074,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F12" s="12" t="s">
         <v>60</v>
       </c>
       <c r="G12" s="19"/>
       <c r="H12" s="19"/>
     </row>
-    <row r="13" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="18" t="s">
         <v>225</v>
       </c>
@@ -2075,14 +2091,14 @@
       <c r="G13" s="19"/>
       <c r="H13" s="19"/>
     </row>
-    <row r="14" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="12" t="s">
         <v>227</v>
       </c>
       <c r="C14" s="19"/>
       <c r="D14" s="19"/>
     </row>
-    <row r="15" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
         <v>228</v>
       </c>
@@ -2100,7 +2116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="20" t="s">
         <v>230</v>
       </c>
@@ -2113,12 +2129,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F17" s="18" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="18" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="18" t="s">
         <v>232</v>
       </c>
@@ -2128,7 +2144,7 @@
       <c r="G18" s="19"/>
       <c r="H18" s="19"/>
     </row>
-    <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="12" t="s">
         <v>234</v>
       </c>
@@ -2140,7 +2156,7 @@
       <c r="G19" s="19"/>
       <c r="H19" s="19"/>
     </row>
-    <row r="20" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="12" t="s">
         <v>236</v>
       </c>
@@ -2158,8 +2174,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="23" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="5" t="s">
         <v>238</v>
       </c>
@@ -2191,7 +2207,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B2:D19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="45" customWidth="1"/>
@@ -2199,17 +2215,17 @@
     <col min="4" max="4" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" ht="23" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="2" spans="2:4" ht="23.1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="14" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="23" t="s">
         <v>242</v>
       </c>
@@ -2220,7 +2236,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="12" t="s">
         <v>245</v>
       </c>
@@ -2229,7 +2245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="12" t="s">
         <v>246</v>
       </c>
@@ -2239,7 +2255,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12" t="s">
         <v>247</v>
       </c>
@@ -2249,7 +2265,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
         <v>248</v>
       </c>
@@ -2259,7 +2275,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="20" t="s">
         <v>249</v>
       </c>
@@ -2272,7 +2288,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="12" t="s">
         <v>250</v>
       </c>
@@ -2282,7 +2298,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="12" t="s">
         <v>251</v>
       </c>
@@ -2292,7 +2308,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="20" t="s">
         <v>252</v>
       </c>
@@ -2305,7 +2321,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="12" t="s">
         <v>253</v>
       </c>
@@ -2315,7 +2331,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
         <v>254</v>
       </c>
@@ -2328,12 +2344,12 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="18" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="12" t="s">
         <v>256</v>
       </c>
@@ -2343,7 +2359,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="20" t="s">
         <v>257</v>
       </c>
@@ -2364,7 +2380,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B2:D32"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
@@ -2372,17 +2388,17 @@
     <col min="4" max="4" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" ht="23" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="2" spans="2:4" ht="23.1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="14" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="23" t="s">
         <v>242</v>
       </c>
@@ -2393,13 +2409,13 @@
         <v>259</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="18" t="s">
         <v>260</v>
       </c>
       <c r="D6" s="15"/>
     </row>
-    <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="12" t="s">
         <v>261</v>
       </c>
@@ -2411,7 +2427,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12" t="s">
         <v>263</v>
       </c>
@@ -2423,13 +2439,13 @@
         <v>262</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="28" t="s">
         <v>264</v>
       </c>
       <c r="D9" s="15"/>
     </row>
-    <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="12" t="s">
         <v>265</v>
       </c>
@@ -2438,7 +2454,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="12" t="s">
         <v>267</v>
       </c>
@@ -2447,7 +2463,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="12" t="s">
         <v>268</v>
       </c>
@@ -2456,7 +2472,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="12" t="s">
         <v>269</v>
       </c>
@@ -2465,7 +2481,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="12" t="s">
         <v>270</v>
       </c>
@@ -2474,7 +2490,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="20" t="s">
         <v>271</v>
       </c>
@@ -2484,7 +2500,7 @@
       </c>
       <c r="D15" s="15"/>
     </row>
-    <row r="16" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
         <v>272</v>
       </c>
@@ -2494,37 +2510,37 @@
       </c>
       <c r="D16" s="15"/>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D17" s="15"/>
     </row>
-    <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="18" t="s">
         <v>273</v>
       </c>
       <c r="D18" s="15"/>
     </row>
-    <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="12" t="s">
         <v>274</v>
       </c>
       <c r="C19" s="19"/>
       <c r="D19" s="15"/>
     </row>
-    <row r="20" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="12" t="s">
         <v>275</v>
       </c>
       <c r="C20" s="19"/>
       <c r="D20" s="15"/>
     </row>
-    <row r="21" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="12" t="s">
         <v>276</v>
       </c>
       <c r="C21" s="19"/>
       <c r="D21" s="15"/>
     </row>
-    <row r="22" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="5" t="s">
         <v>277</v>
       </c>
@@ -2534,51 +2550,51 @@
       </c>
       <c r="D22" s="15"/>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D23" s="15"/>
     </row>
-    <row r="24" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="18" t="s">
         <v>278</v>
       </c>
       <c r="D24" s="15"/>
     </row>
-    <row r="25" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="12" t="s">
         <v>279</v>
       </c>
       <c r="C25" s="19"/>
       <c r="D25" s="15"/>
     </row>
-    <row r="26" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="12" t="s">
         <v>280</v>
       </c>
       <c r="C26" s="19"/>
       <c r="D26" s="15"/>
     </row>
-    <row r="27" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="12" t="s">
         <v>281</v>
       </c>
       <c r="C27" s="19"/>
       <c r="D27" s="15"/>
     </row>
-    <row r="28" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="12" t="s">
         <v>282</v>
       </c>
       <c r="C28" s="19"/>
       <c r="D28" s="15"/>
     </row>
-    <row r="29" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="12" t="s">
         <v>283</v>
       </c>
       <c r="C29" s="19"/>
       <c r="D29" s="15"/>
     </row>
-    <row r="30" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="5" t="s">
         <v>284</v>
       </c>
@@ -2588,10 +2604,10 @@
       </c>
       <c r="D30" s="15"/>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D31" s="15"/>
     </row>
-    <row r="32" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="5" t="s">
         <v>285</v>
       </c>
@@ -2609,7 +2625,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B2:F76"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
@@ -2619,17 +2635,17 @@
     <col min="6" max="6" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="2" spans="2:5" ht="23.1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="14" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="23" t="s">
         <v>2</v>
       </c>
@@ -2643,7 +2659,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="12" t="s">
         <v>6</v>
       </c>
@@ -2655,7 +2671,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="12" t="s">
         <v>8</v>
       </c>
@@ -2670,7 +2686,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12" t="s">
         <v>11</v>
       </c>
@@ -2680,7 +2696,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
         <v>13</v>
       </c>
@@ -2690,7 +2706,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="12" t="s">
         <v>15</v>
       </c>
@@ -2702,7 +2718,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="12" t="s">
         <v>17</v>
       </c>
@@ -2714,7 +2730,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="12" t="s">
         <v>19</v>
       </c>
@@ -2729,15 +2745,15 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B14" s="45" t="s">
+    <row r="14" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="51" t="s">
         <v>22</v>
       </c>
       <c r="C14" s="46"/>
       <c r="D14" s="46"/>
       <c r="E14" s="46"/>
     </row>
-    <row r="15" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
         <v>23</v>
       </c>
@@ -2752,7 +2768,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="12" t="s">
         <v>26</v>
       </c>
@@ -2767,7 +2783,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="12" t="s">
         <v>29</v>
       </c>
@@ -2782,7 +2798,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="12" t="s">
         <v>32</v>
       </c>
@@ -2797,7 +2813,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="12" t="s">
         <v>35</v>
       </c>
@@ -2812,15 +2828,15 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B21" s="45" t="s">
+    <row r="21" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="51" t="s">
         <v>38</v>
       </c>
       <c r="C21" s="46"/>
       <c r="D21" s="46"/>
       <c r="E21" s="46"/>
     </row>
-    <row r="22" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="12" t="s">
         <v>39</v>
       </c>
@@ -2835,7 +2851,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="12" t="s">
         <v>42</v>
       </c>
@@ -2850,7 +2866,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="12" t="s">
         <v>45</v>
       </c>
@@ -2865,7 +2881,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="12" t="s">
         <v>48</v>
       </c>
@@ -2880,7 +2896,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="12" t="s">
         <v>51</v>
       </c>
@@ -2895,7 +2911,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="27" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="12" t="s">
         <v>54</v>
       </c>
@@ -2910,7 +2926,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="28" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="12" t="s">
         <v>57</v>
       </c>
@@ -2925,7 +2941,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="12" t="s">
         <v>60</v>
       </c>
@@ -2940,7 +2956,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="30" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="12" t="s">
         <v>63</v>
       </c>
@@ -2955,7 +2971,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="31" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="12" t="s">
         <v>66</v>
       </c>
@@ -2970,7 +2986,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="12" t="s">
         <v>69</v>
       </c>
@@ -2985,7 +3001,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="33" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="12" t="s">
         <v>72</v>
       </c>
@@ -3000,15 +3016,15 @@
         <v>74</v>
       </c>
     </row>
-    <row r="35" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B35" s="45" t="s">
+    <row r="35" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="51" t="s">
         <v>75</v>
       </c>
       <c r="C35" s="46"/>
       <c r="D35" s="46"/>
       <c r="E35" s="46"/>
     </row>
-    <row r="36" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="12" t="s">
         <v>76</v>
       </c>
@@ -3023,7 +3039,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="37" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="12" t="s">
         <v>79</v>
       </c>
@@ -3038,7 +3054,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="38" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="12" t="s">
         <v>82</v>
       </c>
@@ -3053,7 +3069,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="41" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="23" t="s">
         <v>85</v>
       </c>
@@ -3070,7 +3086,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="42" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="5" t="s">
         <v>89</v>
       </c>
@@ -3078,7 +3094,7 @@
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
     </row>
-    <row r="43" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="12" t="s">
         <v>90</v>
       </c>
@@ -3088,7 +3104,7 @@
       </c>
       <c r="E43" s="30"/>
     </row>
-    <row r="44" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="12" t="s">
         <v>92</v>
       </c>
@@ -3098,7 +3114,7 @@
       </c>
       <c r="E44" s="30"/>
     </row>
-    <row r="45" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="12" t="s">
         <v>94</v>
       </c>
@@ -3108,7 +3124,7 @@
       </c>
       <c r="E45" s="30"/>
     </row>
-    <row r="46" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="46" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="5" t="s">
         <v>96</v>
       </c>
@@ -3116,7 +3132,7 @@
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
     </row>
-    <row r="47" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="12" t="s">
         <v>97</v>
       </c>
@@ -3126,7 +3142,7 @@
       </c>
       <c r="E47" s="30"/>
     </row>
-    <row r="48" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="12" t="s">
         <v>99</v>
       </c>
@@ -3136,7 +3152,7 @@
       </c>
       <c r="E48" s="30"/>
     </row>
-    <row r="49" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="12" t="s">
         <v>101</v>
       </c>
@@ -3146,7 +3162,7 @@
       </c>
       <c r="E49" s="30"/>
     </row>
-    <row r="50" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="50" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="12" t="s">
         <v>103</v>
       </c>
@@ -3156,7 +3172,7 @@
       </c>
       <c r="E50" s="30"/>
     </row>
-    <row r="51" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="12" t="s">
         <v>105</v>
       </c>
@@ -3166,7 +3182,7 @@
       </c>
       <c r="E51" s="30"/>
     </row>
-    <row r="52" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="52" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="12" t="s">
         <v>107</v>
       </c>
@@ -3176,7 +3192,7 @@
       </c>
       <c r="E52" s="30"/>
     </row>
-    <row r="53" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="5" t="s">
         <v>109</v>
       </c>
@@ -3184,7 +3200,7 @@
       <c r="D53" s="1"/>
       <c r="E53" s="1"/>
     </row>
-    <row r="54" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="12" t="s">
         <v>110</v>
       </c>
@@ -3196,7 +3212,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="55" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="12" t="s">
         <v>113</v>
       </c>
@@ -3206,7 +3222,7 @@
       </c>
       <c r="E55" s="30"/>
     </row>
-    <row r="56" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="12" t="s">
         <v>115</v>
       </c>
@@ -3216,7 +3232,7 @@
       </c>
       <c r="E56" s="30"/>
     </row>
-    <row r="57" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="12" t="s">
         <v>117</v>
       </c>
@@ -3226,7 +3242,7 @@
       </c>
       <c r="E57" s="30"/>
     </row>
-    <row r="58" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="58" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="12" t="s">
         <v>119</v>
       </c>
@@ -3236,7 +3252,7 @@
       </c>
       <c r="E58" s="30"/>
     </row>
-    <row r="59" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="59" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="12" t="s">
         <v>121</v>
       </c>
@@ -3246,7 +3262,7 @@
       </c>
       <c r="E59" s="30"/>
     </row>
-    <row r="60" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="12" t="s">
         <v>123</v>
       </c>
@@ -3258,7 +3274,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="61" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="61" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="5" t="s">
         <v>126</v>
       </c>
@@ -3266,7 +3282,7 @@
       <c r="D61" s="1"/>
       <c r="E61" s="1"/>
     </row>
-    <row r="62" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="62" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="12" t="s">
         <v>127</v>
       </c>
@@ -3276,7 +3292,7 @@
       </c>
       <c r="E62" s="30"/>
     </row>
-    <row r="63" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="63" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="12" t="s">
         <v>129</v>
       </c>
@@ -3286,7 +3302,7 @@
       </c>
       <c r="E63" s="30"/>
     </row>
-    <row r="64" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="64" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="12" t="s">
         <v>131</v>
       </c>
@@ -3296,7 +3312,7 @@
       </c>
       <c r="E64" s="30"/>
     </row>
-    <row r="65" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="65" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B65" s="12" t="s">
         <v>133</v>
       </c>
@@ -3306,7 +3322,7 @@
       </c>
       <c r="E65" s="30"/>
     </row>
-    <row r="66" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="66" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B66" s="12" t="s">
         <v>135</v>
       </c>
@@ -3316,7 +3332,7 @@
       </c>
       <c r="E66" s="30"/>
     </row>
-    <row r="67" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="67" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B67" s="12" t="s">
         <v>137</v>
       </c>
@@ -3328,7 +3344,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="68" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="68" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="12" t="s">
         <v>140</v>
       </c>
@@ -3340,7 +3356,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="69" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="69" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B69" s="5" t="s">
         <v>143</v>
       </c>
@@ -3348,7 +3364,7 @@
       <c r="D69" s="1"/>
       <c r="E69" s="1"/>
     </row>
-    <row r="70" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="70" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B70" s="12" t="s">
         <v>144</v>
       </c>
@@ -3358,7 +3374,7 @@
       </c>
       <c r="E70" s="30"/>
     </row>
-    <row r="71" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="71" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B71" s="12" t="s">
         <v>146</v>
       </c>
@@ -3368,7 +3384,7 @@
       </c>
       <c r="E71" s="30"/>
     </row>
-    <row r="72" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="72" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B72" s="12" t="s">
         <v>148</v>
       </c>
@@ -3378,7 +3394,7 @@
       </c>
       <c r="E72" s="30"/>
     </row>
-    <row r="73" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="73" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B73" s="12" t="s">
         <v>150</v>
       </c>
@@ -3388,7 +3404,7 @@
       </c>
       <c r="E73" s="30"/>
     </row>
-    <row r="74" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="74" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B74" s="5" t="s">
         <v>152</v>
       </c>
@@ -3396,7 +3412,7 @@
       <c r="D74" s="1"/>
       <c r="E74" s="1"/>
     </row>
-    <row r="75" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="75" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B75" s="12" t="s">
         <v>153</v>
       </c>
@@ -3410,7 +3426,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="76" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B76" s="12" t="s">
         <v>155</v>
       </c>
@@ -3433,165 +3449,165 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="B2:C24"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.90625" customWidth="1"/>
+    <col min="1" max="1" width="3.85546875" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="23" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="2" spans="2:3" ht="23.1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="14" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B4" s="43" t="s">
         <v>287</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="43" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B5" s="43" t="s">
+      <c r="C5" s="4" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B6" s="43" t="s">
         <v>289</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C6" s="4" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="43" t="s">
         <v>290</v>
       </c>
-    </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B6" s="43" t="s">
+      <c r="C7" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B8" s="43" t="s">
         <v>291</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C8" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B9" s="43" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B7" s="43" t="s">
+      <c r="C9" s="4" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B10" s="43" t="s">
         <v>293</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C10" s="4" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B11" s="43" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B8" s="43" t="s">
+      <c r="C11" s="52" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B12" s="43" t="s">
         <v>295</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B9" s="43" t="s">
+      <c r="C12" s="52" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B13" s="43" t="s">
         <v>296</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C13" s="53" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B14" s="43" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B10" s="43" t="s">
+      <c r="C14" s="53" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B16" s="43" t="s">
         <v>298</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B11" s="43" t="s">
+      <c r="C16" s="4" t="s">
         <v>299</v>
       </c>
-      <c r="C11" s="4" t="s">
+    </row>
+    <row r="17" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="43" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B12" s="43" t="s">
+      <c r="C17" s="4" t="s">
         <v>301</v>
       </c>
-      <c r="C12" s="4" t="s">
+    </row>
+    <row r="18" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="43" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B13" s="43" t="s">
+      <c r="C18" s="4" t="s">
         <v>303</v>
       </c>
-      <c r="C13" s="4" t="s">
+    </row>
+    <row r="19" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="43" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B14" s="43" t="s">
+      <c r="C19" s="4" t="s">
         <v>305</v>
       </c>
-      <c r="C14" s="4" t="s">
+    </row>
+    <row r="20" spans="2:3" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="43" t="s">
         <v>306</v>
       </c>
-    </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B16" s="43" t="s">
+      <c r="C20" s="4" t="s">
         <v>307</v>
       </c>
-      <c r="C16" s="4" t="s">
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B22" s="43" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="43" t="s">
+    <row r="23" spans="2:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="43" t="s">
         <v>309</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C23" s="4" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="43" t="s">
+    <row r="24" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="43" t="s">
         <v>311</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C24" s="4" t="s">
         <v>312</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="43" t="s">
-        <v>313</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="20" spans="2:3" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="43" t="s">
-        <v>315</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B22" s="43" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="23" spans="2:3" ht="32" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="43" t="s">
-        <v>318</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="24" spans="2:3" ht="45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="43" t="s">
-        <v>320</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Completed Balance sheet data
Adding data for Balance sheet only, still some sheet data need to be competed
</commit_message>
<xml_diff>
--- a/models/builds/2026-05-17-cam-sectra-financials.xlsx
+++ b/models/builds/2026-05-17-cam-sectra-financials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\0.BUS Finance\Corporate-Finance\models\builds\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D20585A8-810B-4F25-B611-C4263D13F694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA38F836-04BC-451E-A225-AD5237642BDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1905" yWindow="480" windowWidth="13065" windowHeight="15345" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -127,7 +127,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="337">
   <si>
     <t>Ratios &amp; Derived Inputs</t>
   </si>
@@ -1099,6 +1099,45 @@
   </si>
   <si>
     <t>192.67 million (per Sectra IR / S&amp;P Global; verify FY24/25 Annual Report share note)</t>
+  </si>
+  <si>
+    <t>IFRS-SPECIFIC CONVENTIONS:</t>
+  </si>
+  <si>
+    <t>1. Currency: All figures in SEK Millions unless otherwise stated.</t>
+  </si>
+  <si>
+    <t>2. Fiscal Year: Sectra fiscal year runs May 1 – April 30. FY2024/2025 = May 2024 – April 2025. Care needed when benchmarking against calendar-year peers.</t>
+  </si>
+  <si>
+    <t>3. Deferred Revenue: Sectra reports this as "Contract liabilities" (IFRS 15). When populating BAL_* deferred revenue, use Contract liabilities value (current + non-current).</t>
+  </si>
+  <si>
+    <t>4. Operating Profit Adjustment: FY2024/2025 reported operating profit (SEK 723M) includes SEK 110M non-recurring patent settlement. Underlying operating profit = SEK 613M. Use underlying for like-for-like analysis at Stage 5.</t>
+  </si>
+  <si>
+    <t>5. R&amp;D: Under IAS 38, certain development costs may be capitalized as intangibles rather than expensed. Verify Sectra's policy in accounting notes.</t>
+  </si>
+  <si>
+    <t>6. Translation Effects: Majority revenue (USD/GBP/EUR) translated to SEK at period-average rates. FY2024/2025 marked end of FX tailwinds.</t>
+  </si>
+  <si>
+    <t>7. Tax Rate: Sweden statutory CIT = 20.6%. Sectra effective rate to be calculated from Income Statement.</t>
+  </si>
+  <si>
+    <t>8. IFRS-to-GAAP Mapping:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Receivables (IFRS) ≈ Accounts Receivable (US GAAP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Trade payables ≈ Accounts Payable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Borrowings ≈ Short-term + Long-term Debt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Contract liabilities ≈ Deferred Revenue</t>
   </si>
 </sst>
 </file>
@@ -1115,7 +1154,7 @@
     <numFmt numFmtId="170" formatCode="0.0&quot; days&quot;"/>
     <numFmt numFmtId="171" formatCode="0.000"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1227,6 +1266,14 @@
       <color rgb="FF024731"/>
       <name val="Open Sans"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -1305,7 +1352,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1398,6 +1445,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3448,7 +3496,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="B2:C24"/>
+  <dimension ref="B2:C46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.85546875" customWidth="1"/>
@@ -3610,6 +3658,71 @@
         <v>312</v>
       </c>
     </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B26" s="54" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B38" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B42" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B43" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B46" t="s">
+        <v>336</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update data to Income Statement of the Template
Update data to Income Statement, still need to find Dividends to complete
</commit_message>
<xml_diff>
--- a/models/builds/2026-05-17-cam-sectra-financials.xlsx
+++ b/models/builds/2026-05-17-cam-sectra-financials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\0.BUS Finance\Corporate-Finance\models\builds\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA38F836-04BC-451E-A225-AD5237642BDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A89B00C4-559A-4818-A0F0-A2C9CD3C6E91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1905" yWindow="480" windowWidth="13065" windowHeight="15345" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15480" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -127,7 +127,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="355">
   <si>
     <t>Ratios &amp; Derived Inputs</t>
   </si>
@@ -1138,6 +1138,60 @@
   </si>
   <si>
     <t xml:space="preserve">   - Contract liabilities ≈ Deferred Revenue</t>
+  </si>
+  <si>
+    <t>COGS / GROSS MARGIN LIMITATION (IFRS by-nature reporting):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sectra presents its income statement BY NATURE (IFRS), not BY FUNCTION (US GAAP). </t>
+  </si>
+  <si>
+    <t>It does NOT disclose a "Cost of Goods Sold" or "Gross Profit" line.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- "Cost of goods sold" in this template = "Goods for resale" (SEK 441,712K FY24/25 / </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  431,218K FY23/24) — the cost of hardware Sectra purchases and resells alongside its </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  software systems. This is the ONLY cost line that maps cleanly to COGS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">- As a medical-imaging IT / software company, Sectra's largest true cost is Personnel </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  costs (SEK 1,598,697K FY24/25). A portion of this represents software development, </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  implementation, and support that would be classified as COGS under by-function </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  reporting — but Sectra does not disclose this split, so it cannot be reliably </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  separated and is reported within SG&amp;A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- CONSEQUENCE: The "Gross Margin" ratio computed in this model will appear </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  unusually high (~86%) because most production-related personnel cost sits below </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  the gross-profit line. Gross Margin is therefore NOT meaningful for Sectra and </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  should not be compared to by-function reporters. Operating Margin (EBIT/Sales) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  is the reliable profitability measure here and ties exactly to Sectra's audited </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Operating profit.</t>
   </si>
 </sst>
 </file>
@@ -1432,6 +1486,11 @@
     <xf numFmtId="49" fontId="18" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1441,11 +1500,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1761,33 +1815,33 @@
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="45" t="s">
+    <row r="4" spans="2:3" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="B4" s="48" t="s">
         <v>157</v>
       </c>
-      <c r="C4" s="46"/>
-    </row>
-    <row r="5" spans="2:3" ht="26.1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="49" t="s">
+      <c r="C4" s="49"/>
+    </row>
+    <row r="5" spans="2:3" ht="26.1" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="B5" s="52" t="s">
         <v>158</v>
       </c>
-      <c r="C5" s="46"/>
-    </row>
-    <row r="6" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="47" t="s">
+      <c r="C5" s="49"/>
+    </row>
+    <row r="6" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="50" t="s">
         <v>159</v>
       </c>
-      <c r="C6" s="46"/>
+      <c r="C6" s="49"/>
     </row>
     <row r="7" spans="2:3" ht="3.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
     </row>
     <row r="9" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="48" t="s">
+      <c r="B9" s="51" t="s">
         <v>160</v>
       </c>
-      <c r="C9" s="46"/>
+      <c r="C9" s="49"/>
     </row>
     <row r="10" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
@@ -1838,10 +1892,10 @@
       </c>
     </row>
     <row r="17" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="48" t="s">
+      <c r="B17" s="51" t="s">
         <v>173</v>
       </c>
-      <c r="C17" s="46"/>
+      <c r="C17" s="49"/>
     </row>
     <row r="18" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="5" t="s">
@@ -1851,7 +1905,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="6" t="s">
         <v>176</v>
       </c>
@@ -1859,7 +1913,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="20" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="8" t="s">
         <v>178</v>
       </c>
@@ -1867,7 +1921,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="21" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="9" t="s">
         <v>180</v>
       </c>
@@ -1875,7 +1929,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="22" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="10" t="s">
         <v>182</v>
       </c>
@@ -1884,10 +1938,10 @@
       </c>
     </row>
     <row r="24" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="48" t="s">
+      <c r="B24" s="51" t="s">
         <v>184</v>
       </c>
-      <c r="C24" s="46"/>
+      <c r="C24" s="49"/>
     </row>
     <row r="25" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="5" t="s">
@@ -1962,10 +2016,10 @@
       </c>
     </row>
     <row r="36" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="48" t="s">
+      <c r="B36" s="51" t="s">
         <v>202</v>
       </c>
-      <c r="C36" s="46"/>
+      <c r="C36" s="49"/>
     </row>
     <row r="37" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="12" t="s">
@@ -1984,10 +2038,10 @@
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B41" s="50" t="s">
+      <c r="B41" s="53" t="s">
         <v>207</v>
       </c>
-      <c r="C41" s="46"/>
+      <c r="C41" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -2047,7 +2101,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="18" t="s">
         <v>214</v>
       </c>
@@ -2055,58 +2109,90 @@
         <v>215</v>
       </c>
     </row>
-    <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="12" t="s">
         <v>216</v>
       </c>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
+      <c r="C7" s="19">
+        <v>1341871</v>
+      </c>
+      <c r="D7" s="19">
+        <v>804640</v>
+      </c>
       <c r="F7" s="12" t="s">
         <v>217</v>
       </c>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-    </row>
-    <row r="8" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G7" s="19">
+        <v>23617</v>
+      </c>
+      <c r="H7" s="19">
+        <v>12584</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12" t="s">
         <v>218</v>
       </c>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
+      <c r="C8" s="19">
+        <v>572036</v>
+      </c>
+      <c r="D8" s="19">
+        <v>571661</v>
+      </c>
       <c r="F8" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="G8" s="19"/>
-      <c r="H8" s="19"/>
-    </row>
-    <row r="9" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G8" s="19">
+        <v>107279</v>
+      </c>
+      <c r="H8" s="19">
+        <v>76071</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="12" t="s">
         <v>220</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
+      <c r="C9" s="19">
+        <v>37576</v>
+      </c>
+      <c r="D9" s="19">
+        <v>36590</v>
+      </c>
       <c r="F9" s="12" t="s">
         <v>221</v>
       </c>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
+      <c r="G9" s="19">
+        <f>74321+5619+81667+434012+974935</f>
+        <v>1570554</v>
+      </c>
+      <c r="H9" s="19">
+        <f>67170+2637+75332+408706+946263</f>
+        <v>1500108</v>
+      </c>
     </row>
     <row r="10" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="12" t="s">
         <v>222</v>
       </c>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
+      <c r="C10" s="19">
+        <f>26055+42861+118978+819754</f>
+        <v>1007648</v>
+      </c>
+      <c r="D10" s="19">
+        <f>10274+13354+102610+983019</f>
+        <v>1109257</v>
+      </c>
       <c r="F10" s="20" t="s">
         <v>223</v>
       </c>
       <c r="G10" s="21">
         <f>SUM(G7:G9)</f>
-        <v>0</v>
+        <v>1701450</v>
       </c>
       <c r="H10" s="21">
         <f>SUM(H7:H9)</f>
-        <v>0</v>
+        <v>1588763</v>
       </c>
     </row>
     <row r="11" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2115,19 +2201,23 @@
       </c>
       <c r="C11" s="21">
         <f>SUM(C7:C10)</f>
-        <v>0</v>
+        <v>2959131</v>
       </c>
       <c r="D11" s="21">
         <f>SUM(D7:D10)</f>
-        <v>0</v>
+        <v>2522148</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F12" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="G12" s="19"/>
-      <c r="H12" s="19"/>
+      <c r="G12" s="19">
+        <v>63840</v>
+      </c>
+      <c r="H12" s="19">
+        <v>19204</v>
+      </c>
     </row>
     <row r="13" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="18" t="s">
@@ -2136,15 +2226,25 @@
       <c r="F13" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="G13" s="19"/>
-      <c r="H13" s="19"/>
+      <c r="G13" s="19">
+        <f>58318+4063+11733</f>
+        <v>74114</v>
+      </c>
+      <c r="H13" s="19">
+        <f>26342+7038</f>
+        <v>33380</v>
+      </c>
     </row>
     <row r="14" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="12" t="s">
         <v>227</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
+      <c r="C14" s="19">
+        <v>220654</v>
+      </c>
+      <c r="D14" s="19">
+        <v>227040</v>
+      </c>
     </row>
     <row r="15" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
@@ -2157,11 +2257,11 @@
       </c>
       <c r="G15" s="21">
         <f>G10+G12+G13</f>
-        <v>0</v>
+        <v>1839404</v>
       </c>
       <c r="H15" s="21">
         <f>H10+H12+H13</f>
-        <v>0</v>
+        <v>1641347</v>
       </c>
     </row>
     <row r="16" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2170,11 +2270,11 @@
       </c>
       <c r="C16" s="21">
         <f>C14-C15</f>
-        <v>0</v>
+        <v>220654</v>
       </c>
       <c r="D16" s="21">
         <f>D14-D15</f>
-        <v>0</v>
+        <v>227040</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2189,37 +2289,59 @@
       <c r="F18" s="12" t="s">
         <v>233</v>
       </c>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
+      <c r="G18" s="19">
+        <f>39025+361470</f>
+        <v>400495</v>
+      </c>
+      <c r="H18" s="19">
+        <f>38825+361470</f>
+        <v>400295</v>
+      </c>
     </row>
     <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="12" t="s">
         <v>234</v>
       </c>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
+      <c r="C19" s="19">
+        <v>283063</v>
+      </c>
+      <c r="D19" s="19">
+        <v>262330</v>
+      </c>
       <c r="F19" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
+      <c r="G19" s="19">
+        <f>103919+1412411</f>
+        <v>1516330</v>
+      </c>
+      <c r="H19" s="19">
+        <f>151446+1017850</f>
+        <v>1169296</v>
+      </c>
     </row>
     <row r="20" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="12" t="s">
         <v>236</v>
       </c>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
+      <c r="C20" s="19">
+        <f>106415+126345+32807+19312+8502</f>
+        <v>293381</v>
+      </c>
+      <c r="D20" s="19">
+        <f>35241+138422+21+16746+8990</f>
+        <v>199420</v>
+      </c>
       <c r="F20" s="20" t="s">
         <v>237</v>
       </c>
       <c r="G20" s="21">
         <f>G18+G19</f>
-        <v>0</v>
+        <v>1916825</v>
       </c>
       <c r="H20" s="21">
         <f>H18+H19</f>
-        <v>0</v>
+        <v>1569591</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2229,22 +2351,22 @@
       </c>
       <c r="C23" s="22">
         <f>C11+C16+C19+C20</f>
-        <v>0</v>
+        <v>3756229</v>
       </c>
       <c r="D23" s="22">
         <f>D11+D16+D19+D20</f>
-        <v>0</v>
+        <v>3210938</v>
       </c>
       <c r="F23" s="5" t="s">
         <v>239</v>
       </c>
       <c r="G23" s="22">
         <f>G15+G20</f>
-        <v>0</v>
+        <v>3756229</v>
       </c>
       <c r="H23" s="22">
         <f>H15+H20</f>
-        <v>0</v>
+        <v>3210938</v>
       </c>
     </row>
   </sheetData>
@@ -2268,7 +2390,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.3">
       <c r="B3" s="15" t="s">
         <v>241</v>
       </c>
@@ -2288,7 +2410,9 @@
       <c r="B6" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="C6" s="19"/>
+      <c r="C6" s="19">
+        <v>3239811</v>
+      </c>
       <c r="D6" s="24">
         <v>1</v>
       </c>
@@ -2297,30 +2421,38 @@
       <c r="B7" s="12" t="s">
         <v>246</v>
       </c>
-      <c r="C7" s="19"/>
-      <c r="D7" s="25" t="str">
+      <c r="C7" s="19">
+        <v>441712</v>
+      </c>
+      <c r="D7" s="25">
         <f t="shared" ref="D7:D15" si="0">IFERROR(C7/$C$6,"")</f>
-        <v/>
+        <v>0.13633881729520642</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12" t="s">
         <v>247</v>
       </c>
-      <c r="C8" s="19"/>
-      <c r="D8" s="25" t="str">
+      <c r="C8" s="19">
+        <f>1598697+665324-74093-226356</f>
+        <v>1963572</v>
+      </c>
+      <c r="D8" s="25">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.60607609517962624</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="25" t="str">
+      <c r="C9" s="19">
+        <f>51559+35931+24040</f>
+        <v>111530</v>
+      </c>
+      <c r="D9" s="25">
         <f t="shared" si="0"/>
-        <v/>
+        <v>3.4424847622284142E-2</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2329,31 +2461,35 @@
       </c>
       <c r="C10" s="21">
         <f>C6-C7-C8-C9</f>
-        <v>0</v>
-      </c>
-      <c r="D10" s="25" t="str">
+        <v>722997</v>
+      </c>
+      <c r="D10" s="25">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.22316023990288322</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="12" t="s">
         <v>250</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="25" t="str">
+      <c r="C11" s="19">
+        <v>31404</v>
+      </c>
+      <c r="D11" s="25">
         <f t="shared" si="0"/>
-        <v/>
+        <v>9.693158026810823E-3</v>
       </c>
     </row>
     <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="12" t="s">
         <v>251</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="25" t="str">
+      <c r="C12" s="19">
+        <v>28120</v>
+      </c>
+      <c r="D12" s="25">
         <f t="shared" si="0"/>
-        <v/>
+        <v>8.6795186509336496E-3</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2362,21 +2498,23 @@
       </c>
       <c r="C13" s="21">
         <f>C10+C11-C12</f>
-        <v>0</v>
-      </c>
-      <c r="D13" s="25" t="str">
+        <v>726281</v>
+      </c>
+      <c r="D13" s="25">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.2241738792787604</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="12" t="s">
         <v>253</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="25" t="str">
+      <c r="C14" s="19">
+        <v>162910</v>
+      </c>
+      <c r="D14" s="25">
         <f t="shared" si="0"/>
-        <v/>
+        <v>5.0283797419046976E-2</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2385,11 +2523,11 @@
       </c>
       <c r="C15" s="22">
         <f>C13-C14</f>
-        <v>0</v>
-      </c>
-      <c r="D15" s="26" t="str">
+        <v>563371</v>
+      </c>
+      <c r="D15" s="26">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0.17389008185971341</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2402,9 +2540,9 @@
         <v>256</v>
       </c>
       <c r="C18" s="19"/>
-      <c r="D18" s="25" t="str">
+      <c r="D18" s="25">
         <f>IFERROR(C18/$C$6,"")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2413,11 +2551,11 @@
       </c>
       <c r="C19" s="21">
         <f>C15-C18</f>
-        <v>0</v>
-      </c>
-      <c r="D19" s="25" t="str">
+        <v>563371</v>
+      </c>
+      <c r="D19" s="25">
         <f>IFERROR(C19/$C$6,"")</f>
-        <v/>
+        <v>0.17389008185971341</v>
       </c>
     </row>
   </sheetData>
@@ -2441,7 +2579,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.3">
       <c r="B3" s="15" t="s">
         <v>241</v>
       </c>
@@ -2469,7 +2607,7 @@
       </c>
       <c r="C7" s="27">
         <f>INC_net</f>
-        <v>0</v>
+        <v>563371</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>262</v>
@@ -2481,7 +2619,7 @@
       </c>
       <c r="C8" s="27">
         <f>INC_depreciation</f>
-        <v>0</v>
+        <v>111530</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>262</v>
@@ -2554,7 +2692,7 @@
       </c>
       <c r="C16" s="22">
         <f>C7+C8+C15</f>
-        <v>0</v>
+        <v>674901</v>
       </c>
       <c r="D16" s="15"/>
     </row>
@@ -2661,7 +2799,7 @@
       </c>
       <c r="C32" s="22">
         <f>C16+C22+C30</f>
-        <v>0</v>
+        <v>674901</v>
       </c>
       <c r="D32" s="15"/>
     </row>
@@ -2778,7 +2916,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="12" t="s">
         <v>19</v>
       </c>
@@ -2793,13 +2931,13 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="51" t="s">
+    <row r="14" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="54" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="49"/>
     </row>
     <row r="15" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
@@ -2807,7 +2945,7 @@
       </c>
       <c r="C15" s="36">
         <f>BAL_equity_shareholders_prior</f>
-        <v>0</v>
+        <v>1569591</v>
       </c>
       <c r="D15" s="30" t="s">
         <v>24</v>
@@ -2822,7 +2960,7 @@
       </c>
       <c r="C16" s="36">
         <f>BAL_inventories_prior</f>
-        <v>0</v>
+        <v>36590</v>
       </c>
       <c r="D16" s="30" t="s">
         <v>27</v>
@@ -2837,7 +2975,7 @@
       </c>
       <c r="C17" s="36">
         <f>BAL_receivables_prior</f>
-        <v>0</v>
+        <v>571661</v>
       </c>
       <c r="D17" s="30" t="s">
         <v>30</v>
@@ -2852,7 +2990,7 @@
       </c>
       <c r="C18" s="36">
         <f>BAL_assets_total_prior</f>
-        <v>0</v>
+        <v>3210938</v>
       </c>
       <c r="D18" s="30" t="s">
         <v>33</v>
@@ -2867,7 +3005,7 @@
       </c>
       <c r="C19" s="36">
         <f>BAL_debt_long_term_prior+BAL_equity_shareholders_prior</f>
-        <v>0</v>
+        <v>1588795</v>
       </c>
       <c r="D19" s="30" t="s">
         <v>36</v>
@@ -2876,21 +3014,21 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="51" t="s">
+    <row r="21" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="54" t="s">
         <v>38</v>
       </c>
-      <c r="C21" s="46"/>
-      <c r="D21" s="46"/>
-      <c r="E21" s="46"/>
-    </row>
-    <row r="22" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C21" s="49"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="49"/>
+    </row>
+    <row r="22" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="12" t="s">
         <v>39</v>
       </c>
       <c r="C22" s="36">
         <f>INC_net+(1-tax_rate)*INC_interest_expense</f>
-        <v>0</v>
+        <v>585585.80000000005</v>
       </c>
       <c r="D22" s="30" t="s">
         <v>40</v>
@@ -2905,7 +3043,7 @@
       </c>
       <c r="C23" s="37">
         <f>IFERROR(INC_sales/365,"")</f>
-        <v>0</v>
+        <v>8876.194520547946</v>
       </c>
       <c r="D23" s="30" t="s">
         <v>43</v>
@@ -2920,7 +3058,7 @@
       </c>
       <c r="C24" s="36">
         <f>BAL_equity_shareholders_curr</f>
-        <v>0</v>
+        <v>1916825</v>
       </c>
       <c r="D24" s="30" t="s">
         <v>46</v>
@@ -2935,7 +3073,7 @@
       </c>
       <c r="C25" s="36">
         <f>BAL_cash_marketable_securities_curr</f>
-        <v>0</v>
+        <v>1341871</v>
       </c>
       <c r="D25" s="30" t="s">
         <v>49</v>
@@ -2950,7 +3088,7 @@
       </c>
       <c r="C26" s="36">
         <f>BAL_assets_current_curr</f>
-        <v>0</v>
+        <v>2959131</v>
       </c>
       <c r="D26" s="30" t="s">
         <v>52</v>
@@ -2965,7 +3103,7 @@
       </c>
       <c r="C27" s="36">
         <f>BAL_liabilities_current_curr</f>
-        <v>0</v>
+        <v>1701450</v>
       </c>
       <c r="D27" s="30" t="s">
         <v>55</v>
@@ -2980,7 +3118,7 @@
       </c>
       <c r="C28" s="37">
         <f>IFERROR(INC_cost_goods_sold/365,"")</f>
-        <v>0</v>
+        <v>1210.1698630136987</v>
       </c>
       <c r="D28" s="30" t="s">
         <v>58</v>
@@ -2995,7 +3133,7 @@
       </c>
       <c r="C29" s="36">
         <f>BAL_debt_long_term_curr</f>
-        <v>0</v>
+        <v>63840</v>
       </c>
       <c r="D29" s="30" t="s">
         <v>61</v>
@@ -3004,13 +3142,13 @@
         <v>62</v>
       </c>
     </row>
-    <row r="30" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="12" t="s">
         <v>63</v>
       </c>
       <c r="C30" s="36">
         <f>BAL_assets_current_curr-BAL_liabilities_current_curr</f>
-        <v>0</v>
+        <v>1257681</v>
       </c>
       <c r="D30" s="30" t="s">
         <v>64</v>
@@ -3025,7 +3163,7 @@
       </c>
       <c r="C31" s="36">
         <f>BAL_assets_total_curr</f>
-        <v>0</v>
+        <v>3756229</v>
       </c>
       <c r="D31" s="30" t="s">
         <v>67</v>
@@ -3040,7 +3178,7 @@
       </c>
       <c r="C32" s="36">
         <f>BAL_debt_long_term_curr+BAL_equity_shareholders_curr</f>
-        <v>0</v>
+        <v>1980665</v>
       </c>
       <c r="D32" s="30" t="s">
         <v>70</v>
@@ -3055,7 +3193,7 @@
       </c>
       <c r="C33" s="36">
         <f>BAL_liabilities_total_curr</f>
-        <v>0</v>
+        <v>1839404</v>
       </c>
       <c r="D33" s="30" t="s">
         <v>73</v>
@@ -3064,13 +3202,13 @@
         <v>74</v>
       </c>
     </row>
-    <row r="35" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="51" t="s">
+    <row r="35" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="54" t="s">
         <v>75</v>
       </c>
-      <c r="C35" s="46"/>
-      <c r="D35" s="46"/>
-      <c r="E35" s="46"/>
+      <c r="C35" s="49"/>
+      <c r="D35" s="49"/>
+      <c r="E35" s="49"/>
     </row>
     <row r="36" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="12" t="s">
@@ -3078,7 +3216,7 @@
       </c>
       <c r="C36" s="37">
         <f>AVERAGE(startYear_equity,currentYear_equity)</f>
-        <v>0</v>
+        <v>1743208</v>
       </c>
       <c r="D36" s="30" t="s">
         <v>77</v>
@@ -3093,7 +3231,7 @@
       </c>
       <c r="C37" s="37">
         <f>AVERAGE(startYear_total_assets,currentYear_assets_total)</f>
-        <v>0</v>
+        <v>3483583.5</v>
       </c>
       <c r="D37" s="30" t="s">
         <v>80</v>
@@ -3108,7 +3246,7 @@
       </c>
       <c r="C38" s="37">
         <f>AVERAGE(startYear_total_capitalization,currentYear_total_capitalization)</f>
-        <v>0</v>
+        <v>1784730</v>
       </c>
       <c r="D38" s="30" t="s">
         <v>83</v>
@@ -3142,7 +3280,7 @@
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
     </row>
-    <row r="43" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="12" t="s">
         <v>90</v>
       </c>
@@ -3162,7 +3300,7 @@
       </c>
       <c r="E44" s="30"/>
     </row>
-    <row r="45" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="12" t="s">
         <v>94</v>
       </c>
@@ -3496,7 +3634,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="B2:C46"/>
+  <dimension ref="B2:C68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.85546875" customWidth="1"/>
@@ -3569,7 +3707,7 @@
       <c r="B11" s="43" t="s">
         <v>294</v>
       </c>
-      <c r="C11" s="52" t="s">
+      <c r="C11" s="45" t="s">
         <v>320</v>
       </c>
     </row>
@@ -3577,7 +3715,7 @@
       <c r="B12" s="43" t="s">
         <v>295</v>
       </c>
-      <c r="C12" s="52" t="s">
+      <c r="C12" s="45" t="s">
         <v>321</v>
       </c>
     </row>
@@ -3585,7 +3723,7 @@
       <c r="B13" s="43" t="s">
         <v>296</v>
       </c>
-      <c r="C13" s="53" t="s">
+      <c r="C13" s="46" t="s">
         <v>322</v>
       </c>
     </row>
@@ -3593,7 +3731,7 @@
       <c r="B14" s="43" t="s">
         <v>297</v>
       </c>
-      <c r="C14" s="53" t="s">
+      <c r="C14" s="46" t="s">
         <v>323</v>
       </c>
     </row>
@@ -3659,7 +3797,7 @@
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B26" s="54" t="s">
+      <c r="B26" s="47" t="s">
         <v>324</v>
       </c>
     </row>
@@ -3721,6 +3859,96 @@
     <row r="46" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>336</v>
+      </c>
+    </row>
+    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B48" s="47" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B51" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B54" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B55" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B56" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B57" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B58" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B59" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B60" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B61" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B63" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B65" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B66" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B67" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B68" t="s">
+        <v>354</v>
       </c>
     </row>
   </sheetData>

</xml_diff>